<commit_message>
Format faculty names cleanly with proper spacing and title casing (e.g. M.renuka -> M Renuka)
</commit_message>
<xml_diff>
--- a/Generated_Reports/3rd_Semester_Course_Code_Course_List_with_Faculty_Details.xlsx
+++ b/Generated_Reports/3rd_Semester_Course_Code_Course_List_with_Faculty_Details.xlsx
@@ -546,7 +546,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Roja . Akkaraboyina</t>
+          <t>Roja Akkaraboyina</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -590,7 +590,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Lakshmi Devi. V</t>
+          <t>Lakshmi Devi V</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -665,7 +665,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Kobagapu.likhitha</t>
+          <t>Kobagapu Likhitha</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
@@ -687,7 +687,7 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Kobagapu.likhitha</t>
+          <t>Kobagapu Likhitha</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -709,7 +709,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Kobagapu.likhitha</t>
+          <t>Kobagapu Likhitha</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Kobagapu.likhitha</t>
+          <t>Kobagapu Likhitha</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
@@ -753,7 +753,7 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Dr Adi Seshu Gidugu, Dr.sr.prema Kumari</t>
+          <t>Dr Adi Seshu Gidugu, Dr Sr Prema Kumari</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
@@ -775,7 +775,7 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Dr Adi Seshu Gidugu, Dr.sr.prema Kumari</t>
+          <t>Dr Adi Seshu Gidugu, Dr Sr Prema Kumari</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
@@ -819,7 +819,7 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Dr. L. Anugata</t>
+          <t>Dr L Anugata</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
@@ -841,7 +841,7 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Dr. L. Anugata</t>
+          <t>Dr L Anugata</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
@@ -885,7 +885,7 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>E. P. S. Bhagya Lakshmi</t>
+          <t>E P S Bhagya Lakshmi</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
@@ -938,7 +938,7 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>M.renuka</t>
+          <t>M Renuka</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
@@ -960,7 +960,7 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Lavanya.p</t>
+          <t>Lavanya P</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
@@ -982,7 +982,7 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Dr. Jayasri Puli</t>
+          <t>Dr Jayasri Puli</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
@@ -1026,7 +1026,7 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Y.anasuya Devi</t>
+          <t>Y Anasuya Devi</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
@@ -1101,7 +1101,7 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>V.anjali Devi</t>
+          <t>V Anjali Devi</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>V.anjali Devi</t>
+          <t>V Anjali Devi</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
@@ -1299,7 +1299,7 @@
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>K.kanaka Triveni</t>
+          <t>K Kanaka Triveni</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
@@ -1321,7 +1321,7 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>K.kanaka Triveni</t>
+          <t>K Kanaka Triveni</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>E. P. S. Bhagya Lakshmi</t>
+          <t>E P S Bhagya Lakshmi</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Lavanya.p</t>
+          <t>Lavanya P</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
@@ -1440,7 +1440,7 @@
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Lavanya.p</t>
+          <t>Lavanya P</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>A.divya Jyothi</t>
+          <t>A Divya Jyothi</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
@@ -1528,7 +1528,7 @@
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>Y.anasuya Devi</t>
+          <t>Y Anasuya Devi</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
@@ -1691,7 +1691,7 @@
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>V. Kavitha</t>
+          <t>V Kavitha</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>E. P. S. Bhagya Lakshmi</t>
+          <t>E P S Bhagya Lakshmi</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
@@ -1757,7 +1757,7 @@
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>E. P. S. Bhagya Lakshmi</t>
+          <t>E P S Bhagya Lakshmi</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
@@ -2030,7 +2030,7 @@
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>K.kanaka Triveni</t>
+          <t>K Kanaka Triveni</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
@@ -2052,7 +2052,7 @@
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>K.kanaka Triveni</t>
+          <t>K Kanaka Triveni</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
@@ -2074,7 +2074,7 @@
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>Y.anasuya Devi</t>
+          <t>Y Anasuya Devi</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>E. P. S. Bhagya Lakshmi</t>
+          <t>E P S Bhagya Lakshmi</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
@@ -2325,7 +2325,7 @@
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>K.kanaka Triveni</t>
+          <t>K Kanaka Triveni</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
@@ -2347,7 +2347,7 @@
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>K.kanaka Triveni</t>
+          <t>K Kanaka Triveni</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
@@ -2391,7 +2391,7 @@
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>E. P. S. Bhagya Lakshmi</t>
+          <t>E P S Bhagya Lakshmi</t>
         </is>
       </c>
       <c r="D101" s="5" t="inlineStr">
@@ -2466,7 +2466,7 @@
       </c>
       <c r="C106" s="4" t="inlineStr">
         <is>
-          <t>Dr. Ch. Prasanthi, Dr. L. Anugata</t>
+          <t>Dr Ch Prasanthi, Dr L Anugata</t>
         </is>
       </c>
       <c r="D106" s="5" t="inlineStr">
@@ -2488,7 +2488,7 @@
       </c>
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t>Dr. Ch. Prasanthi</t>
+          <t>Dr Ch Prasanthi</t>
         </is>
       </c>
       <c r="D107" s="5" t="inlineStr">
@@ -2510,7 +2510,7 @@
       </c>
       <c r="C108" s="4" t="inlineStr">
         <is>
-          <t>Dr. Ch. Prasanthi</t>
+          <t>Dr Ch Prasanthi</t>
         </is>
       </c>
       <c r="D108" s="5" t="inlineStr">
@@ -2532,7 +2532,7 @@
       </c>
       <c r="C109" s="4" t="inlineStr">
         <is>
-          <t>Dr. L. Anugata</t>
+          <t>Dr L Anugata</t>
         </is>
       </c>
       <c r="D109" s="5" t="inlineStr">
@@ -2554,7 +2554,7 @@
       </c>
       <c r="C110" s="4" t="inlineStr">
         <is>
-          <t>Dr. L. Anugata</t>
+          <t>Dr L Anugata</t>
         </is>
       </c>
       <c r="D110" s="5" t="inlineStr">
@@ -2576,7 +2576,7 @@
       </c>
       <c r="C111" s="4" t="inlineStr">
         <is>
-          <t>Dr. L. Anugata</t>
+          <t>Dr L Anugata</t>
         </is>
       </c>
       <c r="D111" s="5" t="inlineStr">
@@ -2598,7 +2598,7 @@
       </c>
       <c r="C112" s="4" t="inlineStr">
         <is>
-          <t>Dr. L. Anugata</t>
+          <t>Dr L Anugata</t>
         </is>
       </c>
       <c r="D112" s="5" t="inlineStr">
@@ -2730,7 +2730,7 @@
       </c>
       <c r="C118" s="4" t="inlineStr">
         <is>
-          <t>E. P. S. Bhagya Lakshmi</t>
+          <t>E P S Bhagya Lakshmi</t>
         </is>
       </c>
       <c r="D118" s="5" t="inlineStr">
@@ -2805,7 +2805,7 @@
       </c>
       <c r="C123" s="4" t="inlineStr">
         <is>
-          <t>Roja . Akkaraboyina</t>
+          <t>Roja Akkaraboyina</t>
         </is>
       </c>
       <c r="D123" s="5" t="inlineStr">
@@ -3166,7 +3166,7 @@
       </c>
       <c r="C141" s="4" t="inlineStr">
         <is>
-          <t>E. P. S. Bhagya Lakshmi</t>
+          <t>E P S Bhagya Lakshmi</t>
         </is>
       </c>
       <c r="D141" s="5" t="inlineStr">

</xml_diff>